<commit_message>
Reset Excel Table for LATHE-01
</commit_message>
<xml_diff>
--- a/FM-MN-07_LATHE-01.xlsx
+++ b/FM-MN-07_LATHE-01.xlsx
@@ -1715,17 +1715,9 @@
           <t>การ WORM SPINDLE ก่อนเริ่มงาน 15 นาที</t>
         </is>
       </c>
-      <c r="C6" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="44" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E6" s="44" t="inlineStr"/>
       <c r="F6" s="7" t="inlineStr"/>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr"/>
@@ -1764,17 +1756,9 @@
           <t>เช็คระดับน้ำมันเครื่องในห้องเกียร์</t>
         </is>
       </c>
-      <c r="C7" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="44" t="inlineStr"/>
       <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E7" s="44" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr"/>
@@ -1813,17 +1797,9 @@
           <t>เช็คระบบเฟื่องทดลองเปลี่ยนรอบตวามเร็วต่าง ๆ</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="44" t="inlineStr"/>
       <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E8" s="44" t="inlineStr"/>
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr"/>
@@ -1862,17 +1838,9 @@
           <t>เช็ค AUTO แกน X,Y</t>
         </is>
       </c>
-      <c r="C9" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="44" t="inlineStr"/>
       <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E9" s="44" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
       <c r="G9" s="7" t="inlineStr"/>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1911,17 +1879,9 @@
           <t>เช็คระดับน้ำมันหล่อลื่นใน PUMP</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="44" t="inlineStr"/>
       <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E10" s="44" t="inlineStr"/>
       <c r="F10" s="7" t="inlineStr"/>
       <c r="G10" s="7" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1960,17 +1920,9 @@
           <t>เช็คน้ำมันหล่อเย็นและการทำงานของปั้ม</t>
         </is>
       </c>
-      <c r="C11" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C11" s="44" t="inlineStr"/>
       <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E11" s="44" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr"/>
       <c r="G11" s="7" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr"/>
@@ -2009,17 +1961,9 @@
           <t>ตรวจสอบหน้าจอ  DIGITAL  READ OUT และการ ทำงานของ  LINEAR  SCALE</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C12" s="45" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr"/>
-      <c r="E12" s="45" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E12" s="45" t="inlineStr"/>
       <c r="F12" s="11" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr"/>
       <c r="H12" s="11" t="inlineStr"/>
@@ -2058,17 +2002,9 @@
           <t>ตรวจเช็คสภาพและความตึงของสายพาน</t>
         </is>
       </c>
-      <c r="C13" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C13" s="44" t="inlineStr"/>
       <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E13" s="44" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr"/>
       <c r="G13" s="7" t="inlineStr"/>
       <c r="H13" s="7" t="inlineStr"/>
@@ -2107,17 +2043,9 @@
           <t>ตรวจสอบการทำงานของไฟฟ้าแสงสว่าง</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C14" s="44" t="inlineStr"/>
       <c r="D14" s="7" t="inlineStr"/>
-      <c r="E14" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E14" s="44" t="inlineStr"/>
       <c r="F14" s="7" t="inlineStr"/>
       <c r="G14" s="7" t="inlineStr"/>
       <c r="H14" s="7" t="inlineStr"/>
@@ -2156,17 +2084,9 @@
           <t>อัดจาระบีตามหัวอัดจาระบีทุก ๆ จุด</t>
         </is>
       </c>
-      <c r="C15" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C15" s="44" t="inlineStr"/>
       <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E15" s="44" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr"/>
@@ -2205,17 +2125,9 @@
           <t>ตรวจสอบความพร้อมสภาพโดยรวมของเครื่อง</t>
         </is>
       </c>
-      <c r="C16" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C16" s="44" t="inlineStr"/>
       <c r="D16" s="7" t="inlineStr"/>
-      <c r="E16" s="44" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E16" s="44" t="inlineStr"/>
       <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="7" t="inlineStr"/>
       <c r="H16" s="7" t="inlineStr"/>
@@ -2248,17 +2160,9 @@
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="5" t="n"/>
-      <c r="C17" s="46" t="inlineStr">
-        <is>
-          <t>ลุงคอง</t>
-        </is>
-      </c>
+      <c r="C17" s="46" t="inlineStr"/>
       <c r="D17" s="41" t="inlineStr"/>
-      <c r="E17" s="46" t="inlineStr">
-        <is>
-          <t>ขวัญชัย</t>
-        </is>
-      </c>
+      <c r="E17" s="46" t="inlineStr"/>
       <c r="F17" s="41" t="inlineStr"/>
       <c r="G17" s="41" t="inlineStr"/>
       <c r="H17" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for LATHE-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_LATHE-01.xlsx
+++ b/FM-MN-07_LATHE-01.xlsx
@@ -1720,7 +1720,11 @@
       <c r="E6" s="44" t="inlineStr"/>
       <c r="F6" s="7" t="inlineStr"/>
       <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="H6" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="7" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
@@ -1761,7 +1765,11 @@
       <c r="E7" s="44" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
+      <c r="H7" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
@@ -1802,7 +1810,11 @@
       <c r="E8" s="44" t="inlineStr"/>
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
+      <c r="H8" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
@@ -1843,7 +1855,11 @@
       <c r="E9" s="44" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
       <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
+      <c r="H9" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="7" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
@@ -1884,7 +1900,11 @@
       <c r="E10" s="44" t="inlineStr"/>
       <c r="F10" s="7" t="inlineStr"/>
       <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
+      <c r="H10" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="7" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
@@ -1925,7 +1945,11 @@
       <c r="E11" s="44" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr"/>
       <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
+      <c r="H11" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="7" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
@@ -1966,7 +1990,11 @@
       <c r="E12" s="45" t="inlineStr"/>
       <c r="F12" s="11" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr"/>
-      <c r="H12" s="11" t="inlineStr"/>
+      <c r="H12" s="45" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="11" t="inlineStr"/>
@@ -2007,7 +2035,11 @@
       <c r="E13" s="44" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr"/>
       <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
+      <c r="H13" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
@@ -2048,7 +2080,11 @@
       <c r="E14" s="44" t="inlineStr"/>
       <c r="F14" s="7" t="inlineStr"/>
       <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="H14" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="7" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
@@ -2089,7 +2125,11 @@
       <c r="E15" s="44" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="H15" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="7" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
@@ -2130,7 +2170,11 @@
       <c r="E16" s="44" t="inlineStr"/>
       <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="H16" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="7" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr"/>
@@ -2165,7 +2209,11 @@
       <c r="E17" s="46" t="inlineStr"/>
       <c r="F17" s="41" t="inlineStr"/>
       <c r="G17" s="41" t="inlineStr"/>
-      <c r="H17" s="41" t="inlineStr"/>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>ลุงคอง</t>
+        </is>
+      </c>
       <c r="I17" s="41" t="inlineStr"/>
       <c r="J17" s="41" t="inlineStr"/>
       <c r="K17" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for LATHE-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_LATHE-01.xlsx
+++ b/FM-MN-07_LATHE-01.xlsx
@@ -1725,7 +1725,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr"/>
+      <c r="I6" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="7" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="7" t="inlineStr"/>
@@ -1770,7 +1774,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
@@ -1815,7 +1823,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
@@ -1860,7 +1872,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="7" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
@@ -1905,7 +1921,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="I10" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="7" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
@@ -1950,7 +1970,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="I11" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="7" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
@@ -1995,7 +2019,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr"/>
+      <c r="I12" s="45" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="11" t="inlineStr"/>
       <c r="L12" s="11" t="inlineStr"/>
@@ -2040,7 +2068,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="I13" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="7" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
       <c r="L13" s="7" t="inlineStr"/>
@@ -2085,7 +2117,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J14" s="7" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr"/>
@@ -2130,7 +2166,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="I15" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J15" s="7" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
@@ -2175,7 +2215,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="I16" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J16" s="7" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="7" t="inlineStr"/>
@@ -2214,7 +2258,11 @@
           <t>ลุงคอง</t>
         </is>
       </c>
-      <c r="I17" s="41" t="inlineStr"/>
+      <c r="I17" s="46" t="inlineStr">
+        <is>
+          <t>ลุงคอง</t>
+        </is>
+      </c>
       <c r="J17" s="41" t="inlineStr"/>
       <c r="K17" s="41" t="inlineStr"/>
       <c r="L17" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for LATHE-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_LATHE-01.xlsx
+++ b/FM-MN-07_LATHE-01.xlsx
@@ -1733,7 +1733,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr"/>
+      <c r="J6" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="7" t="inlineStr"/>
       <c r="M6" s="7" t="inlineStr"/>
@@ -1782,7 +1786,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr"/>
+      <c r="J7" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr"/>
@@ -1831,7 +1839,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr"/>
+      <c r="J8" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
       <c r="M8" s="7" t="inlineStr"/>
@@ -1880,7 +1892,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr"/>
+      <c r="J9" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr"/>
@@ -1929,7 +1945,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr"/>
+      <c r="J10" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
       <c r="M10" s="7" t="inlineStr"/>
@@ -1978,7 +1998,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr"/>
+      <c r="J11" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="7" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
       <c r="M11" s="7" t="inlineStr"/>
@@ -2027,7 +2051,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr"/>
+      <c r="J12" s="45" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="11" t="inlineStr"/>
       <c r="L12" s="11" t="inlineStr"/>
       <c r="M12" s="11" t="inlineStr"/>
@@ -2076,7 +2104,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr"/>
+      <c r="J13" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="7" t="inlineStr"/>
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr"/>
@@ -2125,7 +2157,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr"/>
+      <c r="J14" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr"/>
       <c r="M14" s="7" t="inlineStr"/>
@@ -2174,7 +2210,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr"/>
+      <c r="J15" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr"/>
@@ -2223,7 +2263,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr"/>
+      <c r="J16" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="7" t="inlineStr"/>
       <c r="M16" s="7" t="inlineStr"/>
@@ -2266,7 +2310,11 @@
           <t>ลุงคอง</t>
         </is>
       </c>
-      <c r="J17" s="41" t="inlineStr"/>
+      <c r="J17" s="46" t="inlineStr">
+        <is>
+          <t>ลุงคอง</t>
+        </is>
+      </c>
       <c r="K17" s="41" t="inlineStr"/>
       <c r="L17" s="41" t="inlineStr"/>
       <c r="M17" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for LATHE-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_LATHE-01.xlsx
+++ b/FM-MN-07_LATHE-01.xlsx
@@ -1739,7 +1739,11 @@
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr"/>
-      <c r="L6" s="7" t="inlineStr"/>
+      <c r="L6" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="7" t="inlineStr"/>
       <c r="N6" s="7" t="inlineStr"/>
       <c r="O6" s="7" t="inlineStr"/>
@@ -1792,7 +1796,11 @@
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="inlineStr"/>
       <c r="O7" s="7" t="inlineStr"/>
@@ -1845,7 +1853,11 @@
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="L8" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="7" t="inlineStr"/>
       <c r="N8" s="7" t="inlineStr"/>
       <c r="O8" s="7" t="inlineStr"/>
@@ -1898,7 +1910,11 @@
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="7" t="inlineStr"/>
       <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="inlineStr"/>
@@ -1951,7 +1967,11 @@
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="L10" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="7" t="inlineStr"/>
       <c r="N10" s="7" t="inlineStr"/>
       <c r="O10" s="7" t="inlineStr"/>
@@ -2004,7 +2024,11 @@
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="inlineStr"/>
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr"/>
@@ -2057,7 +2081,11 @@
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="11" t="inlineStr"/>
+      <c r="L12" s="45" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="11" t="inlineStr"/>
       <c r="N12" s="11" t="inlineStr"/>
       <c r="O12" s="11" t="inlineStr"/>
@@ -2110,7 +2138,11 @@
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="L13" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="inlineStr"/>
       <c r="N13" s="7" t="inlineStr"/>
       <c r="O13" s="7" t="inlineStr"/>
@@ -2163,7 +2195,11 @@
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr"/>
-      <c r="L14" s="7" t="inlineStr"/>
+      <c r="L14" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="7" t="inlineStr"/>
       <c r="N14" s="7" t="inlineStr"/>
       <c r="O14" s="7" t="inlineStr"/>
@@ -2216,7 +2252,11 @@
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="7" t="inlineStr"/>
       <c r="N15" s="7" t="inlineStr"/>
       <c r="O15" s="7" t="inlineStr"/>
@@ -2269,7 +2309,11 @@
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr"/>
-      <c r="L16" s="7" t="inlineStr"/>
+      <c r="L16" s="44" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="7" t="inlineStr"/>
       <c r="N16" s="7" t="inlineStr"/>
       <c r="O16" s="7" t="inlineStr"/>
@@ -2316,7 +2360,11 @@
         </is>
       </c>
       <c r="K17" s="41" t="inlineStr"/>
-      <c r="L17" s="41" t="inlineStr"/>
+      <c r="L17" s="46" t="inlineStr">
+        <is>
+          <t>ลุงคอง</t>
+        </is>
+      </c>
       <c r="M17" s="41" t="inlineStr"/>
       <c r="N17" s="41" t="inlineStr"/>
       <c r="O17" s="41" t="inlineStr"/>

</xml_diff>